<commit_message>
Benchmark quality and consistency update
</commit_message>
<xml_diff>
--- a/participant/18_bank_and_payment_records.xlsx
+++ b/participant/18_bank_and_payment_records.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rc66a79480b1d49e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Statement" sheetId="2" r:id="R864250356e9f49af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Ledger" sheetId="3" r:id="R4655b0c6a0e2482c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="4" r:id="R8557dd545ce04db7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R6f93314dbe8a4448"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Raf18d1997f50484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Statement" sheetId="2" r:id="R23afcfc722e64df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Ledger" sheetId="3" r:id="R952479167df14973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="4" r:id="Rfde12e60066840e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="Rde4a9ee760ba4570"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -709,7 +709,7 @@
         <x:v>Record scope</x:v>
       </x:c>
       <x:c r="B14" s="33" t="str">
-        <x:v>Condensed but complete in aggregate; ordinary operating transactions are grouped</x:v>
+        <x:v>Condensed extract, not a complete statement; selected transactions are shown and omitted debits and credits are represented only by a net as-of reconciliation adjustment</x:v>
       </x:c>
       <x:c r="C14" s="33"/>
       <x:c r="D14" s="33"/>
@@ -735,7 +735,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="36" t="str">
-        <x:v>Evidence limitations: the statement rows are a synthetic bank export. The participant file does not include bank officer certification, complete mandate forms, source SWIFT/NEFT messages or the Riverstone diligence mandate. One bank reference differs by one digit from the internal ledger; categories and approval records also conflict.</x:v>
+        <x:v>Evidence limitations: the rows are a synthetic selected bank export, not a complete statement. The participant file does not include bank officer certification, complete mandate forms, source SWIFT/NEFT messages, the gross composition or timing of omitted movements, or the Riverstone diligence mandate. One bank reference differs by one digit from the internal ledger; categories and approval records also conflict. VP-05 records unaudited cash of INR 38.6m on 7 August, while this selected-row reconstruction shows INR 44.9m; the basis, cutoff and any restriction classification are unresolved.</x:v>
       </x:c>
       <x:c r="B16" s="36"/>
       <x:c r="C16" s="36"/>
@@ -823,7 +823,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="32" t="str">
-        <x:v>Account ending 4419 | Values in INR | Condensed statement; ordinary operating transactions are aggregated</x:v>
+        <x:v>Account ending 4419 | Values in INR | Selected extract, not a complete statement; reconciliation adjustments do not establish transaction timing or gross flows</x:v>
       </x:c>
       <x:c r="B2" s="32"/>
       <x:c r="C2" s="32"/>
@@ -863,7 +863,7 @@
         <x:v>Credit</x:v>
       </x:c>
       <x:c r="G4" s="46" t="str">
-        <x:v>Running balance</x:v>
+        <x:v>Selected-row reconstruction</x:v>
       </x:c>
       <x:c r="H4" s="47" t="str">
         <x:v>Counterparty</x:v>
@@ -1193,29 +1193,29 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="48" t="n">
-        <x:v>45905</x:v>
+        <x:v>45909</x:v>
       </x:c>
       <x:c r="B17" s="48" t="n">
-        <x:v>45905</x:v>
+        <x:v>45909</x:v>
       </x:c>
       <x:c r="C17" s="33" t="str">
-        <x:v>OPS-AGG-APRSEP</x:v>
+        <x:v>CLOUDSEP</x:v>
       </x:c>
       <x:c r="D17" s="33" t="str">
-        <x:v>ORDINARY OPERATING PAYMENTS - AGGREGATED</x:v>
+        <x:v>CLOUD AND INFRASTRUCTURE</x:v>
       </x:c>
       <x:c r="E17" s="35" t="n">
-        <x:v>12200000</x:v>
+        <x:v>6100000</x:v>
       </x:c>
       <x:c r="F17" s="35" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="35" t="n">
         <x:f>G16+F17-E17</x:f>
-        <x:v>19500000</x:v>
+        <x:v>25600000</x:v>
       </x:c>
       <x:c r="H17" s="33" t="str">
-        <x:v>Multiple counterparties</x:v>
+        <x:v>Multiple vendors</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1226,13 +1226,13 @@
         <x:v>45909</x:v>
       </x:c>
       <x:c r="C18" s="33" t="str">
-        <x:v>CLOUDSEP</x:v>
+        <x:v>RECON-OMITTED-TO-0909</x:v>
       </x:c>
       <x:c r="D18" s="33" t="str">
-        <x:v>CLOUD AND INFRASTRUCTURE</x:v>
+        <x:v>NET OMITTED MOVEMENTS - AS-OF 9 SEP</x:v>
       </x:c>
       <x:c r="E18" s="35" t="n">
-        <x:v>6100000</x:v>
+        <x:v>12200000</x:v>
       </x:c>
       <x:c r="F18" s="35" t="n">
         <x:v>0</x:v>
@@ -1242,7 +1242,7 @@
         <x:v>13400000</x:v>
       </x:c>
       <x:c r="H18" s="33" t="str">
-        <x:v>Multiple vendors</x:v>
+        <x:v>Multiple / unidentified</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2287,7 +2287,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="33" t="str">
-        <x:v>Running balance final</x:v>
+        <x:v>Reconstructed closing balance</x:v>
       </x:c>
       <x:c r="B10" s="35" t="n">
         <x:f>'Bank Statement'!G24</x:f>
@@ -2305,14 +2305,14 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F10" s="33" t="str">
-        <x:v>Condensed statement ties from opening balance through all aggregate movements</x:v>
+        <x:v>Selected rows plus the net as-of adjustment reconcile the reported closing figure; this does not establish completeness, timing or gross flows</x:v>
       </x:c>
       <x:c r="G10" s="33"/>
       <x:c r="H10" s="33"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="33" t="str">
-        <x:v>Unrestricted cash at 9 Sep</x:v>
+        <x:v>Reported unrestricted cash at 9 Sep</x:v>
       </x:c>
       <x:c r="B11" s="35" t="n">
         <x:f>'Bank Statement'!G18</x:f>
@@ -2330,7 +2330,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F11" s="33" t="str">
-        <x:v>Matches VP-10 after aggregated ordinary operating payments</x:v>
+        <x:v>Selected rows plus the net as-of adjustment reconcile VP-10; omitted gross movements and timing remain unknown</x:v>
       </x:c>
       <x:c r="G11" s="33"/>
       <x:c r="H11" s="33"/>
@@ -2360,23 +2360,49 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
+        <x:v>7 Aug cash discrepancy</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:f>'Bank Statement'!G15</x:f>
+        <x:v>44900000</x:v>
+      </x:c>
+      <x:c r="C13" t="n">
+        <x:v>38600000</x:v>
+      </x:c>
+      <x:c r="D13" t="n">
+        <x:f>B13-C13</x:f>
+        <x:v>6300000</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>REVIEW</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>VP-05 records CFO unaudited cash of INR 38.6m; this reconstruction shows INR 44.9m. Basis, cutoff and restriction classification are unresolved.</x:v>
+      </x:c>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
         <x:v>Formula error scan</x:v>
       </x:c>
-      <x:c r="B13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="B14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="F14" t="str">
         <x:v>No spreadsheet formula errors intended</x:v>
       </x:c>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>